<commit_message>
Update BGDPbES file with latest US data.
</commit_message>
<xml_diff>
--- a/InputData/elec/BGDPbES/BAU Guaranteed Dispatch Perc by Elec Source.xlsx
+++ b/InputData/elec/BGDPbES/BAU Guaranteed Dispatch Perc by Elec Source.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25330"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11027"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\elec\BGDPbES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/elec/BGDPbES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E73A0787-3581-4D21-A9CD-91111CFCA519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE007FB5-0C6B-3741-B9CF-FB23EB2FC914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4300" yWindow="780" windowWidth="19420" windowHeight="10420" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -1165,9 +1165,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1205,9 +1205,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1240,26 +1240,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1292,26 +1275,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1486,14 +1452,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>326</v>
       </c>
@@ -1501,67 +1467,67 @@
         <v>327</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B4" s="4">
         <v>2022</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>347</v>
       </c>
@@ -1575,28 +1541,28 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAB677FF-8AA7-4A99-AA5C-83E52BC9397F}">
   <dimension ref="A1:BB120"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="42.6328125" customWidth="1"/>
-    <col min="23" max="23" width="51.36328125" customWidth="1"/>
+    <col min="1" max="1" width="42.6640625" customWidth="1"/>
+    <col min="23" max="23" width="51.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -1607,7 +1573,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="5" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -1663,7 +1629,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="6" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>26</v>
       </c>
@@ -1677,7 +1643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>35</v>
       </c>
@@ -1691,7 +1657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>36</v>
       </c>
@@ -1852,7 +1818,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="9" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>40</v>
       </c>
@@ -2013,7 +1979,7 @@
         <v>404.52</v>
       </c>
     </row>
-    <row r="10" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>43</v>
       </c>
@@ -2174,7 +2140,7 @@
         <v>1588.52</v>
       </c>
     </row>
-    <row r="11" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>46</v>
       </c>
@@ -2323,7 +2289,7 @@
         <v>644.45500000000004</v>
       </c>
     </row>
-    <row r="12" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>49</v>
       </c>
@@ -2484,7 +2450,7 @@
         <v>281.92700000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>52</v>
       </c>
@@ -2645,7 +2611,7 @@
         <v>1304.52</v>
       </c>
     </row>
-    <row r="14" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>55</v>
       </c>
@@ -2806,7 +2772,7 @@
         <v>1147.81</v>
       </c>
     </row>
-    <row r="15" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>58</v>
       </c>
@@ -2967,7 +2933,7 @@
         <v>5.53383</v>
       </c>
     </row>
-    <row r="16" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>61</v>
       </c>
@@ -3128,7 +3094,7 @@
         <v>22.668299999999999</v>
       </c>
     </row>
-    <row r="17" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>64</v>
       </c>
@@ -3277,7 +3243,7 @@
         <v>22.699000000000002</v>
       </c>
     </row>
-    <row r="18" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>67</v>
       </c>
@@ -3438,7 +3404,7 @@
         <v>12.764900000000001</v>
       </c>
     </row>
-    <row r="19" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>70</v>
       </c>
@@ -3587,7 +3553,7 @@
         <v>381.23099999999999</v>
       </c>
     </row>
-    <row r="20" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>73</v>
       </c>
@@ -3748,7 +3714,7 @@
         <v>33.837800000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>76</v>
       </c>
@@ -3909,7 +3875,7 @@
         <v>45.145099999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>79</v>
       </c>
@@ -4019,7 +3985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>36</v>
       </c>
@@ -4156,7 +4122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>40</v>
       </c>
@@ -4293,7 +4259,7 @@
         <v>16.524899999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>43</v>
       </c>
@@ -4334,7 +4300,7 @@
         <v>26.24</v>
       </c>
     </row>
-    <row r="26" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>49</v>
       </c>
@@ -4375,7 +4341,7 @@
         <v>7.18</v>
       </c>
     </row>
-    <row r="27" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>88</v>
       </c>
@@ -4416,7 +4382,7 @@
         <v>12.12</v>
       </c>
     </row>
-    <row r="28" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>91</v>
       </c>
@@ -4457,7 +4423,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="29" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>94</v>
       </c>
@@ -4498,7 +4464,7 @@
         <v>103.4</v>
       </c>
     </row>
-    <row r="30" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>97</v>
       </c>
@@ -4539,7 +4505,7 @@
         <v>119.9</v>
       </c>
     </row>
-    <row r="31" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>100</v>
       </c>
@@ -4553,7 +4519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:54" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -4594,7 +4560,7 @@
         <v>58.31</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>40</v>
       </c>
@@ -4635,7 +4601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>43</v>
       </c>
@@ -4676,7 +4642,7 @@
         <v>27.1</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>49</v>
       </c>
@@ -4717,7 +4683,7 @@
         <v>29.67</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>88</v>
       </c>
@@ -4758,7 +4724,7 @@
         <v>10.27</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>91</v>
       </c>
@@ -4799,7 +4765,7 @@
         <v>1.19</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>94</v>
       </c>
@@ -4840,7 +4806,7 @@
         <v>126.54</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>97</v>
       </c>
@@ -4881,7 +4847,7 @@
         <v>149.18</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>116</v>
       </c>
@@ -4895,7 +4861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>36</v>
       </c>
@@ -4936,7 +4902,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>40</v>
       </c>
@@ -4977,7 +4943,7 @@
         <v>148.47999999999999</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>43</v>
       </c>
@@ -5018,7 +4984,7 @@
         <v>276.52</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>49</v>
       </c>
@@ -5059,7 +5025,7 @@
         <v>9.07</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>88</v>
       </c>
@@ -5100,7 +5066,7 @@
         <v>53.43</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>91</v>
       </c>
@@ -5141,7 +5107,7 @@
         <v>1.86</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>94</v>
       </c>
@@ -5182,7 +5148,7 @@
         <v>822.36</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>97</v>
       </c>
@@ -5223,7 +5189,7 @@
         <v>781.21</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>132</v>
       </c>
@@ -5237,7 +5203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>36</v>
       </c>
@@ -5278,7 +5244,7 @@
         <v>272.36</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>40</v>
       </c>
@@ -5319,7 +5285,7 @@
         <v>144.88</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>43</v>
       </c>
@@ -5360,7 +5326,7 @@
         <v>223.85</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>49</v>
       </c>
@@ -5401,7 +5367,7 @@
         <v>35.06</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>88</v>
       </c>
@@ -5442,7 +5408,7 @@
         <v>26.22</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>91</v>
       </c>
@@ -5483,7 +5449,7 @@
         <v>-0.78</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>94</v>
       </c>
@@ -5524,7 +5490,7 @@
         <v>701.59</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>97</v>
       </c>
@@ -5565,7 +5531,7 @@
         <v>684.99</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>148</v>
       </c>
@@ -5579,7 +5545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>36</v>
       </c>
@@ -5620,7 +5586,7 @@
         <v>162.52000000000001</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>40</v>
       </c>
@@ -5661,7 +5627,7 @@
         <v>14.42</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>43</v>
       </c>
@@ -5702,7 +5668,7 @@
         <v>29.14</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>49</v>
       </c>
@@ -5743,7 +5709,7 @@
         <v>0.18</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>88</v>
       </c>
@@ -5784,7 +5750,7 @@
         <v>15.69</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>91</v>
       </c>
@@ -5825,7 +5791,7 @@
         <v>2.91</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>94</v>
       </c>
@@ -5866,7 +5832,7 @@
         <v>224.86</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>97</v>
       </c>
@@ -5907,7 +5873,7 @@
         <v>231.36</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>164</v>
       </c>
@@ -5921,7 +5887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>36</v>
       </c>
@@ -5962,7 +5928,7 @@
         <v>181.09</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>40</v>
       </c>
@@ -6003,7 +5969,7 @@
         <v>245.47</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>43</v>
       </c>
@@ -6044,7 +6010,7 @@
         <v>89.67</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>49</v>
       </c>
@@ -6085,7 +6051,7 @@
         <v>10.130000000000001</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>88</v>
       </c>
@@ -6126,7 +6092,7 @@
         <v>111.85</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>91</v>
       </c>
@@ -6167,7 +6133,7 @@
         <v>5.62</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>94</v>
       </c>
@@ -6208,7 +6174,7 @@
         <v>643.83000000000004</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>97</v>
       </c>
@@ -6249,7 +6215,7 @@
         <v>669.87</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>180</v>
       </c>
@@ -6263,7 +6229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>36</v>
       </c>
@@ -6304,7 +6270,7 @@
         <v>55.63</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>40</v>
       </c>
@@ -6345,7 +6311,7 @@
         <v>84.57</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>43</v>
       </c>
@@ -6386,7 +6352,7 @@
         <v>17.350000000000001</v>
       </c>
     </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>49</v>
       </c>
@@ -6427,7 +6393,7 @@
         <v>16.34</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>88</v>
       </c>
@@ -6468,7 +6434,7 @@
         <v>114.53</v>
       </c>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>91</v>
       </c>
@@ -6509,7 +6475,7 @@
         <v>0.64</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>94</v>
       </c>
@@ -6550,7 +6516,7 @@
         <v>289.05</v>
       </c>
     </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>97</v>
       </c>
@@ -6591,7 +6557,7 @@
         <v>275.11</v>
       </c>
     </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>196</v>
       </c>
@@ -6605,7 +6571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>36</v>
       </c>
@@ -6646,7 +6612,7 @@
         <v>132.21</v>
       </c>
     </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>40</v>
       </c>
@@ -6687,7 +6653,7 @@
         <v>74.959999999999994</v>
       </c>
     </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>43</v>
       </c>
@@ -6728,7 +6694,7 @@
         <v>40.83</v>
       </c>
     </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>49</v>
       </c>
@@ -6769,7 +6735,7 @@
         <v>0.62</v>
       </c>
     </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>88</v>
       </c>
@@ -6810,7 +6776,7 @@
         <v>149.37</v>
       </c>
     </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>91</v>
       </c>
@@ -6851,7 +6817,7 @@
         <v>1.35</v>
       </c>
     </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>94</v>
       </c>
@@ -6892,7 +6858,7 @@
         <v>399.34</v>
       </c>
     </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>97</v>
       </c>
@@ -6933,7 +6899,7 @@
         <v>399.34</v>
       </c>
     </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>212</v>
       </c>
@@ -6947,7 +6913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>36</v>
       </c>
@@ -6988,7 +6954,7 @@
         <v>88.52</v>
       </c>
     </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>40</v>
       </c>
@@ -7029,7 +6995,7 @@
         <v>79.459999999999994</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>43</v>
       </c>
@@ -7070,7 +7036,7 @@
         <v>8.35</v>
       </c>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>49</v>
       </c>
@@ -7111,7 +7077,7 @@
         <v>132.16999999999999</v>
       </c>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>88</v>
       </c>
@@ -7152,7 +7118,7 @@
         <v>75.56</v>
       </c>
     </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>91</v>
       </c>
@@ -7193,7 +7159,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>94</v>
       </c>
@@ -7234,7 +7200,7 @@
         <v>384.66</v>
       </c>
     </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>97</v>
       </c>
@@ -7275,7 +7241,7 @@
         <v>359.59</v>
       </c>
     </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>228</v>
       </c>
@@ -7289,7 +7255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>36</v>
       </c>
@@ -7330,7 +7296,7 @@
         <v>44.98</v>
       </c>
     </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>40</v>
       </c>
@@ -7371,7 +7337,7 @@
         <v>21.24</v>
       </c>
     </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>43</v>
       </c>
@@ -7412,7 +7378,7 @@
         <v>31.97</v>
       </c>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>49</v>
       </c>
@@ -7453,7 +7419,7 @@
         <v>8.73</v>
       </c>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>88</v>
       </c>
@@ -7494,7 +7460,7 @@
         <v>21.48</v>
       </c>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>91</v>
       </c>
@@ -7535,7 +7501,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>94</v>
       </c>
@@ -7576,7 +7542,7 @@
         <v>128.55000000000001</v>
       </c>
     </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>97</v>
       </c>
@@ -7617,7 +7583,7 @@
         <v>105.92</v>
       </c>
     </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>244</v>
       </c>
@@ -7631,7 +7597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>36</v>
       </c>
@@ -7672,7 +7638,7 @@
         <v>74.19</v>
       </c>
     </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>40</v>
       </c>
@@ -7713,7 +7679,7 @@
         <v>6.92</v>
       </c>
     </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>43</v>
       </c>
@@ -7754,7 +7720,7 @@
         <v>17.96</v>
       </c>
     </row>
-    <row r="116" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>49</v>
       </c>
@@ -7795,7 +7761,7 @@
         <v>22.77</v>
       </c>
     </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>88</v>
       </c>
@@ -7836,7 +7802,7 @@
         <v>83.26</v>
       </c>
     </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>91</v>
       </c>
@@ -7877,7 +7843,7 @@
         <v>0.17</v>
       </c>
     </row>
-    <row r="119" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>94</v>
       </c>
@@ -7918,7 +7884,7 @@
         <v>205.27</v>
       </c>
     </row>
-    <row r="120" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>97</v>
       </c>
@@ -7967,12 +7933,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5E568DE-48BA-4A53-AD96-D707A1A92561}">
   <dimension ref="A1:AF17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="55.453125" customWidth="1"/>
+    <col min="1" max="1" width="55.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>260</v>
       </c>
@@ -8070,7 +8036,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>261</v>
       </c>
@@ -8168,7 +8134,7 @@
         <v>102.188</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>262</v>
       </c>
@@ -8266,7 +8232,7 @@
         <v>331.03</v>
       </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>263</v>
       </c>
@@ -8364,7 +8330,7 @@
         <v>78.619</v>
       </c>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>264</v>
       </c>
@@ -8462,7 +8428,7 @@
         <v>78.998999999999995</v>
       </c>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>265</v>
       </c>
@@ -8560,7 +8526,7 @@
         <v>325.39400000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>266</v>
       </c>
@@ -8658,7 +8624,7 @@
         <v>429.08699999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>267</v>
       </c>
@@ -8756,7 +8722,7 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>268</v>
       </c>
@@ -8854,7 +8820,7 @@
         <v>5.0869999999999997</v>
       </c>
     </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>269</v>
       </c>
@@ -8952,7 +8918,7 @@
         <v>3.403</v>
       </c>
     </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>270</v>
       </c>
@@ -9050,7 +9016,7 @@
         <v>26.716000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>271</v>
       </c>
@@ -9148,7 +9114,7 @@
         <v>305.649</v>
       </c>
     </row>
-    <row r="13" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>272</v>
       </c>
@@ -9246,7 +9212,7 @@
         <v>6.798</v>
       </c>
     </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>273</v>
       </c>
@@ -9344,7 +9310,7 @@
         <v>8.0239999999999991</v>
       </c>
     </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>274</v>
       </c>
@@ -9442,7 +9408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>275</v>
       </c>
@@ -9540,7 +9506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>276</v>
       </c>
@@ -9646,12 +9612,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94F4A00D-FEE1-4109-9021-DF78FFA4A8D5}">
   <dimension ref="A1:AF49"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="63.26953125" customWidth="1"/>
+    <col min="1" max="1" width="63.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>260</v>
       </c>
@@ -9749,7 +9715,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>277</v>
       </c>
@@ -9847,7 +9813,7 @@
         <v>3854.4</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>278</v>
       </c>
@@ -9945,7 +9911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>279</v>
       </c>
@@ -10043,7 +10009,7 @@
         <v>4239.84</v>
       </c>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>280</v>
       </c>
@@ -10141,7 +10107,7 @@
         <v>7884</v>
       </c>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>281</v>
       </c>
@@ -10239,7 +10205,7 @@
         <v>7884</v>
       </c>
     </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>282</v>
       </c>
@@ -10337,7 +10303,7 @@
         <v>7884</v>
       </c>
     </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>283</v>
       </c>
@@ -10435,7 +10401,7 @@
         <v>8094.24</v>
       </c>
     </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>284</v>
       </c>
@@ -10533,7 +10499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>285</v>
       </c>
@@ -10631,7 +10597,7 @@
         <v>8094.24</v>
       </c>
     </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>286</v>
       </c>
@@ -10729,7 +10695,7 @@
         <v>3565.32</v>
       </c>
     </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>287</v>
       </c>
@@ -10827,7 +10793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>288</v>
       </c>
@@ -10925,7 +10891,7 @@
         <v>3924.48</v>
       </c>
     </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>289</v>
       </c>
@@ -11023,7 +10989,7 @@
         <v>3022.18</v>
       </c>
     </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>290</v>
       </c>
@@ -11121,7 +11087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>291</v>
       </c>
@@ -11219,7 +11185,7 @@
         <v>3809.83</v>
       </c>
     </row>
-    <row r="17" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>292</v>
       </c>
@@ -11317,7 +11283,7 @@
         <v>1999.24</v>
       </c>
     </row>
-    <row r="18" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>293</v>
       </c>
@@ -11415,7 +11381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>294</v>
       </c>
@@ -11513,7 +11479,7 @@
         <v>2362.7399999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>295</v>
       </c>
@@ -11611,7 +11577,7 @@
         <v>1804.56</v>
       </c>
     </row>
-    <row r="21" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>296</v>
       </c>
@@ -11709,7 +11675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>297</v>
       </c>
@@ -11807,7 +11773,7 @@
         <v>5045.76</v>
       </c>
     </row>
-    <row r="23" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>298</v>
       </c>
@@ -11905,7 +11871,7 @@
         <v>7577.4</v>
       </c>
     </row>
-    <row r="24" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>299</v>
       </c>
@@ -12003,7 +11969,7 @@
         <v>7577.4</v>
       </c>
     </row>
-    <row r="25" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>300</v>
       </c>
@@ -12101,7 +12067,7 @@
         <v>7577.4</v>
       </c>
     </row>
-    <row r="26" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>301</v>
       </c>
@@ -12199,7 +12165,7 @@
         <v>6053.16</v>
       </c>
     </row>
-    <row r="27" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>302</v>
       </c>
@@ -12297,7 +12263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>303</v>
       </c>
@@ -12395,7 +12361,7 @@
         <v>6657.6</v>
       </c>
     </row>
-    <row r="29" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>304</v>
       </c>
@@ -12493,7 +12459,7 @@
         <v>490.56</v>
       </c>
     </row>
-    <row r="30" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>305</v>
       </c>
@@ -12591,7 +12557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>306</v>
       </c>
@@ -12689,7 +12655,7 @@
         <v>543.12</v>
       </c>
     </row>
-    <row r="32" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>307</v>
       </c>
@@ -12787,7 +12753,7 @@
         <v>1165.08</v>
       </c>
     </row>
-    <row r="33" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>308</v>
       </c>
@@ -12885,7 +12851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>309</v>
       </c>
@@ -12983,7 +12949,7 @@
         <v>1278.96</v>
       </c>
     </row>
-    <row r="35" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>310</v>
       </c>
@@ -13081,7 +13047,7 @@
         <v>6640.08</v>
       </c>
     </row>
-    <row r="36" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>311</v>
       </c>
@@ -13179,7 +13145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>312</v>
       </c>
@@ -13277,7 +13243,7 @@
         <v>7305.84</v>
       </c>
     </row>
-    <row r="38" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>313</v>
       </c>
@@ -13375,7 +13341,7 @@
         <v>4309.92</v>
       </c>
     </row>
-    <row r="39" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>314</v>
       </c>
@@ -13473,7 +13439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>315</v>
       </c>
@@ -13571,7 +13537,7 @@
         <v>4958.16</v>
       </c>
     </row>
-    <row r="41" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>316</v>
       </c>
@@ -13669,7 +13635,7 @@
         <v>490.56</v>
       </c>
     </row>
-    <row r="42" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>317</v>
       </c>
@@ -13767,7 +13733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>318</v>
       </c>
@@ -13865,7 +13831,7 @@
         <v>543.12</v>
       </c>
     </row>
-    <row r="44" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>319</v>
       </c>
@@ -13963,7 +13929,7 @@
         <v>490.56</v>
       </c>
     </row>
-    <row r="45" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>320</v>
       </c>
@@ -14061,7 +14027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>321</v>
       </c>
@@ -14159,7 +14125,7 @@
         <v>543.12</v>
       </c>
     </row>
-    <row r="47" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>322</v>
       </c>
@@ -14257,7 +14223,7 @@
         <v>7884</v>
       </c>
     </row>
-    <row r="48" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>323</v>
       </c>
@@ -14355,7 +14321,7 @@
         <v>7884</v>
       </c>
     </row>
-    <row r="49" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>324</v>
       </c>
@@ -14461,12 +14427,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2F2634-68D9-4A99-92F0-3688E66AA3CB}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.08984375" customWidth="1"/>
+    <col min="1" max="1" width="23.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B1">
         <v>2020</v>
       </c>
@@ -14474,7 +14440,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>325</v>
       </c>
@@ -14487,7 +14453,7 @@
         <v>1.0000010797726713</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -14500,7 +14466,7 @@
         <v>1.0000010797726713</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="58" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>350</v>
       </c>
@@ -14508,7 +14474,7 @@
         <v>0.92500000000000004</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="58" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>350</v>
       </c>
@@ -14527,13 +14493,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AK17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" customWidth="1"/>
-    <col min="2" max="2" width="11.26953125" customWidth="1"/>
+    <col min="1" max="1" width="23.5" customWidth="1"/>
+    <col min="2" max="2" width="11.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:37" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>25</v>
       </c>
@@ -14646,7 +14612,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -14666,12 +14632,10 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <f>'2020 Calculations'!B2</f>
-        <v>0.82698597951865516</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <f>'2020 Calculations'!C2</f>
-        <v>1.0000010797726713</v>
+        <v>0</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -14789,7 +14753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -14930,7 +14894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -15071,7 +15035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -15212,7 +15176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -15353,7 +15317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -15494,7 +15458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -15635,7 +15599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -15776,7 +15740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -15917,7 +15881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -16058,7 +16022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -16202,7 +16166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -16222,12 +16186,10 @@
         <v>0</v>
       </c>
       <c r="G13">
-        <f>'2020 Calculations'!B3</f>
-        <v>0.71523111742153966</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <f>'2020 Calculations'!C3</f>
-        <v>1.0000010797726713</v>
+        <v>0</v>
       </c>
       <c r="I13">
         <v>0</v>
@@ -16345,7 +16307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -16485,7 +16447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -16598,7 +16560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -16711,7 +16673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>24</v>
       </c>

</xml_diff>